<commit_message>
Update plot to fit thesis page size
</commit_message>
<xml_diff>
--- a/1_analysis/manual_plot/组态.xlsx
+++ b/1_analysis/manual_plot/组态.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ezri/ezridb/forR/20250714_MPA_QCA/1_analysis/manual_plot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07AD2DD8-6B17-214E-8B1B-7E8C9F173AC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5AB087C-ED6F-254E-8469-61721DD826EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="920" yWindow="500" windowWidth="32300" windowHeight="18460" xr2:uid="{8604267B-1582-9548-9AB0-E29EB2750A1D}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="103">
   <si>
     <t>X1</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -650,19 +650,6 @@
         <family val="3"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">风险承担者与投资者	</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
       <t>研发投入</t>
     </r>
   </si>
@@ -675,7 +662,57 @@
         <family val="3"/>
         <charset val="134"/>
       </rPr>
-      <t>研究与试验发展（</t>
+      <t>风险承担者与投资者</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>政府引导基金投资密度</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>风险承担者与投资者</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>政府创新补助</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>上市公司年报财务报表附注</t>
     </r>
     <r>
       <rPr>
@@ -684,79 +721,17 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>R&amp;D)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>经费投入强度</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>风险承担者与投资者</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>政府引导基金投资密度</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>风险承担者与投资者</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>政府创新补助</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>上市公司年报财务报表附注</t>
+      <t>“</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>营业外收入</t>
     </r>
     <r>
       <rPr>
@@ -765,17 +740,17 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>“</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>营业外收入</t>
+      <t>”</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>科目下</t>
     </r>
     <r>
       <rPr>
@@ -784,17 +759,17 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>”</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>科目下</t>
+      <t>“</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>政府补助明细</t>
     </r>
     <r>
       <rPr>
@@ -803,25 +778,6 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>“</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>政府补助明细</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
       <t>”</t>
     </r>
   </si>
@@ -907,18 +863,6 @@
         <family val="3"/>
         <charset val="134"/>
       </rPr>
-      <t>政府创新采购</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
       <t>政府单位创新采购数量对数</t>
     </r>
   </si>
@@ -944,74 +888,7 @@
         <family val="3"/>
         <charset val="134"/>
       </rPr>
-      <t>培养科技人员</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>研究与试验发展（</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>R&amp;D)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>人员全时当量</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>培育创新型企业</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
       <t>高新技术企业数量</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>知识产权保护强度</t>
     </r>
   </si>
   <si>
@@ -1184,6 +1061,106 @@
       </rPr>
       <t>支持</t>
     </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>知识产权保护</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>研究与试验发展（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>R&amp;D</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="SimSun"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>人员全时当量</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>研究与试验发展（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>R&amp;D</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="SimSun"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>经费投入强度</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>政府创新采购</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>培育科技人员</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>培育创新型企业</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1375,7 +1352,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1488,6 +1465,18 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1499,9 +1488,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1851,8 +1837,8 @@
   <cols>
     <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="65.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="56.6640625" customWidth="1"/>
+    <col min="4" max="4" width="19" customWidth="1"/>
     <col min="5" max="5" width="3.33203125" customWidth="1"/>
     <col min="9" max="9" width="2.1640625" customWidth="1"/>
   </cols>
@@ -1874,11 +1860,11 @@
       <c r="C2" s="16"/>
       <c r="D2" s="16"/>
       <c r="E2" s="16"/>
-      <c r="F2" s="38" t="s">
+      <c r="F2" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="38"/>
-      <c r="H2" s="38"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
       <c r="I2" s="16"/>
       <c r="J2" s="20" t="s">
         <v>14</v>
@@ -1889,13 +1875,13 @@
         <v>68</v>
       </c>
       <c r="B3" s="36" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="C3" s="36" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="D3" s="37" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="E3" s="34"/>
       <c r="F3" s="30" t="s">
@@ -1914,13 +1900,13 @@
     </row>
     <row r="4" spans="1:10" ht="25" customHeight="1">
       <c r="A4" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="B4" s="21" t="s">
-        <v>70</v>
-      </c>
-      <c r="C4" s="16" t="s">
-        <v>71</v>
+      <c r="C4" s="40" t="s">
+        <v>99</v>
       </c>
       <c r="D4" s="16" t="s">
         <v>0</v>
@@ -1941,13 +1927,13 @@
     </row>
     <row r="5" spans="1:10" ht="25" customHeight="1">
       <c r="A5" s="21" t="s">
-        <v>72</v>
-      </c>
-      <c r="B5" s="42" t="s">
-        <v>103</v>
+        <v>70</v>
+      </c>
+      <c r="B5" s="38" t="s">
+        <v>96</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D5" s="16" t="s">
         <v>1</v>
@@ -1959,13 +1945,13 @@
     </row>
     <row r="6" spans="1:10" ht="25" customHeight="1">
       <c r="A6" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" s="16" t="s">
         <v>74</v>
-      </c>
-      <c r="B6" s="21" t="s">
-        <v>75</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>76</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>2</v>
@@ -1983,13 +1969,13 @@
     </row>
     <row r="7" spans="1:10" ht="25" customHeight="1">
       <c r="A7" s="21" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="16" t="s">
         <v>77</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>78</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>79</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>47</v>
@@ -2010,13 +1996,13 @@
     </row>
     <row r="8" spans="1:10" ht="25" customHeight="1">
       <c r="A8" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="C8" s="16" t="s">
         <v>80</v>
-      </c>
-      <c r="B8" s="21" t="s">
-        <v>81</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>82</v>
       </c>
       <c r="D8" s="16" t="s">
         <v>48</v>
@@ -2037,13 +2023,13 @@
     </row>
     <row r="9" spans="1:10" ht="25" customHeight="1">
       <c r="A9" s="21" t="s">
-        <v>77</v>
-      </c>
-      <c r="B9" s="21" t="s">
-        <v>83</v>
+        <v>75</v>
+      </c>
+      <c r="B9" s="41" t="s">
+        <v>100</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D9" s="16" t="s">
         <v>49</v>
@@ -2058,13 +2044,13 @@
     </row>
     <row r="10" spans="1:10" ht="25" customHeight="1">
       <c r="A10" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="B10" s="21" t="s">
-        <v>86</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>87</v>
+        <v>82</v>
+      </c>
+      <c r="B10" s="41" t="s">
+        <v>101</v>
+      </c>
+      <c r="C10" s="40" t="s">
+        <v>98</v>
       </c>
       <c r="D10" s="16" t="s">
         <v>50</v>
@@ -2085,13 +2071,13 @@
     </row>
     <row r="11" spans="1:10" ht="25" customHeight="1">
       <c r="A11" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>88</v>
+        <v>82</v>
+      </c>
+      <c r="B11" s="41" t="s">
+        <v>102</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="D11" s="16" t="s">
         <v>51</v>
@@ -2112,13 +2098,13 @@
     </row>
     <row r="12" spans="1:10" ht="25" customHeight="1">
       <c r="A12" s="30" t="s">
-        <v>85</v>
-      </c>
-      <c r="B12" s="30" t="s">
-        <v>90</v>
+        <v>82</v>
+      </c>
+      <c r="B12" s="39" t="s">
+        <v>97</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="D12" s="31" t="s">
         <v>3</v>
@@ -2143,7 +2129,7 @@
         <v>13</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="E13" s="23"/>
       <c r="F13" s="17">
@@ -2191,7 +2177,7 @@
         <v>29</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="E15" s="23"/>
       <c r="F15" s="17">
@@ -2215,7 +2201,7 @@
         <v>28</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="E16" s="23"/>
       <c r="F16" s="17">
@@ -2239,7 +2225,7 @@
         <v>8</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="E17" s="23"/>
       <c r="F17" s="17">
@@ -2263,7 +2249,7 @@
         <v>9</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="E18" s="23"/>
       <c r="F18" s="17">
@@ -2287,14 +2273,14 @@
         <v>10</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="E19" s="23"/>
-      <c r="F19" s="39">
+      <c r="F19" s="43">
         <v>0.98547774549460898</v>
       </c>
-      <c r="G19" s="39"/>
-      <c r="H19" s="39"/>
+      <c r="G19" s="43"/>
+      <c r="H19" s="43"/>
       <c r="I19" s="16"/>
       <c r="J19" s="17">
         <v>0.98369724348282883</v>
@@ -2307,14 +2293,14 @@
         <v>11</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="E20" s="23"/>
-      <c r="F20" s="39">
+      <c r="F20" s="43">
         <v>0.964637475960332</v>
       </c>
-      <c r="G20" s="39"/>
-      <c r="H20" s="39"/>
+      <c r="G20" s="43"/>
+      <c r="H20" s="43"/>
       <c r="I20" s="16"/>
       <c r="J20" s="17">
         <v>0.96913673569809566</v>
@@ -2327,14 +2313,14 @@
         <v>30</v>
       </c>
       <c r="D21" s="26" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="E21" s="26"/>
-      <c r="F21" s="40">
+      <c r="F21" s="44">
         <v>0.61986484810942799</v>
       </c>
-      <c r="G21" s="40"/>
-      <c r="H21" s="40"/>
+      <c r="G21" s="44"/>
+      <c r="H21" s="44"/>
       <c r="I21" s="19"/>
       <c r="J21" s="18">
         <v>0.60970676731688356</v>
@@ -2391,7 +2377,7 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="70" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup paperSize="9" scale="74" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -2411,13 +2397,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
     </row>
     <row r="2" spans="1:11" ht="17" thickBot="1">
       <c r="B2" s="1"/>
@@ -2668,18 +2654,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="45" t="s">
         <v>60</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
     </row>
     <row r="3" spans="1:9" ht="17" thickBot="1">
       <c r="A3" s="1"/>
@@ -2836,11 +2822,11 @@
     </row>
     <row r="10" spans="1:9" ht="17" thickTop="1"/>
     <row r="12" spans="1:9">
-      <c r="A12" s="41" t="s">
+      <c r="A12" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="B12" s="41"/>
-      <c r="C12" s="41"/>
+      <c r="B12" s="45"/>
+      <c r="C12" s="45"/>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" s="2"/>

</xml_diff>